<commit_message>
Separated receiving a message and deserializing it in Receiver class
</commit_message>
<xml_diff>
--- a/time_measurements.xlsx
+++ b/time_measurements.xlsx
@@ -108,7 +108,7 @@
         <v>1.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>0.0</v>
+        <v>1.066672E7</v>
       </c>
     </row>
     <row r="3">
@@ -122,7 +122,7 @@
         <v>5.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>0.0</v>
+        <v>7684900.0</v>
       </c>
     </row>
     <row r="4">
@@ -136,7 +136,7 @@
         <v>10.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>0.0</v>
+        <v>1.08428E7</v>
       </c>
     </row>
     <row r="5">
@@ -150,7 +150,7 @@
         <v>1.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>0.0</v>
+        <v>6.138806E7</v>
       </c>
     </row>
     <row r="6">
@@ -164,7 +164,7 @@
         <v>5.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>0.0</v>
+        <v>5.400424E7</v>
       </c>
     </row>
     <row r="7">
@@ -178,7 +178,7 @@
         <v>10.0</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>0.0</v>
+        <v>5.572194E7</v>
       </c>
     </row>
     <row r="8">
@@ -192,7 +192,7 @@
         <v>1.0</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>0.0</v>
+        <v>6912420.0</v>
       </c>
     </row>
     <row r="9">
@@ -206,7 +206,7 @@
         <v>5.0</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>0.0</v>
+        <v>3053180.0</v>
       </c>
     </row>
     <row r="10">
@@ -220,7 +220,7 @@
         <v>10.0</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>0.0</v>
+        <v>9517080.0</v>
       </c>
     </row>
     <row r="11">
@@ -234,7 +234,7 @@
         <v>1.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>0.0</v>
+        <v>1859100.0</v>
       </c>
     </row>
     <row r="12">
@@ -248,7 +248,7 @@
         <v>5.0</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>0.0</v>
+        <v>3861780.0</v>
       </c>
     </row>
     <row r="13">
@@ -262,7 +262,7 @@
         <v>10.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>0.0</v>
+        <v>4818400.0</v>
       </c>
     </row>
     <row r="14">
@@ -276,7 +276,7 @@
         <v>1.0</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>0.0</v>
+        <v>5501040.0</v>
       </c>
     </row>
     <row r="15">
@@ -290,7 +290,7 @@
         <v>5.0</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>0.0</v>
+        <v>1.051218E7</v>
       </c>
     </row>
     <row r="16">
@@ -304,7 +304,7 @@
         <v>10.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>0.0</v>
+        <v>9492460.0</v>
       </c>
     </row>
     <row r="17">
@@ -318,7 +318,7 @@
         <v>1.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>0.0</v>
+        <v>1.200218E7</v>
       </c>
     </row>
     <row r="18">
@@ -332,7 +332,7 @@
         <v>5.0</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>0.0</v>
+        <v>2147200.0</v>
       </c>
     </row>
     <row r="19">
@@ -346,7 +346,7 @@
         <v>10.0</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>0.0</v>
+        <v>5194440.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Everything works juuuuust fine
</commit_message>
<xml_diff>
--- a/time_measurements.xlsx
+++ b/time_measurements.xlsx
@@ -108,7 +108,7 @@
         <v>1.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>1.066672E7</v>
+        <v>4.121808E7</v>
       </c>
     </row>
     <row r="3">
@@ -122,7 +122,7 @@
         <v>5.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>7684900.0</v>
+        <v>4.07036E7</v>
       </c>
     </row>
     <row r="4">
@@ -136,7 +136,7 @@
         <v>10.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>1.08428E7</v>
+        <v>4.638378E7</v>
       </c>
     </row>
     <row r="5">
@@ -150,7 +150,7 @@
         <v>1.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>6.138806E7</v>
+        <v>3.437449E8</v>
       </c>
     </row>
     <row r="6">
@@ -164,7 +164,7 @@
         <v>5.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>5.400424E7</v>
+        <v>3.4291622E8</v>
       </c>
     </row>
     <row r="7">
@@ -178,7 +178,7 @@
         <v>10.0</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>5.572194E7</v>
+        <v>3.5122836E8</v>
       </c>
     </row>
     <row r="8">
@@ -192,7 +192,7 @@
         <v>1.0</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>6912420.0</v>
+        <v>1.285362E7</v>
       </c>
     </row>
     <row r="9">
@@ -206,7 +206,7 @@
         <v>5.0</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>3053180.0</v>
+        <v>7041560.0</v>
       </c>
     </row>
     <row r="10">
@@ -220,7 +220,7 @@
         <v>10.0</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>9517080.0</v>
+        <v>2.157416E7</v>
       </c>
     </row>
     <row r="11">
@@ -234,7 +234,7 @@
         <v>1.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>1859100.0</v>
+        <v>3229440.0</v>
       </c>
     </row>
     <row r="12">
@@ -248,7 +248,7 @@
         <v>5.0</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>3861780.0</v>
+        <v>6560880.0</v>
       </c>
     </row>
     <row r="13">
@@ -262,7 +262,7 @@
         <v>10.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>4818400.0</v>
+        <v>3878960.0</v>
       </c>
     </row>
     <row r="14">
@@ -276,7 +276,7 @@
         <v>1.0</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>5501040.0</v>
+        <v>2.913706E7</v>
       </c>
     </row>
     <row r="15">
@@ -290,7 +290,7 @@
         <v>5.0</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>1.051218E7</v>
+        <v>4.707114E7</v>
       </c>
     </row>
     <row r="16">
@@ -304,7 +304,7 @@
         <v>10.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>9492460.0</v>
+        <v>4.95406E7</v>
       </c>
     </row>
     <row r="17">
@@ -318,7 +318,7 @@
         <v>1.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>1.200218E7</v>
+        <v>1.210302E7</v>
       </c>
     </row>
     <row r="18">
@@ -332,7 +332,7 @@
         <v>5.0</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>2147200.0</v>
+        <v>2001880.0</v>
       </c>
     </row>
     <row r="19">
@@ -346,7 +346,7 @@
         <v>10.0</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>5194440.0</v>
+        <v>3227240.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ready for time measurement
</commit_message>
<xml_diff>
--- a/time_measurements.xlsx
+++ b/time_measurements.xlsx
@@ -102,13 +102,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C2" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>4.121808E7</v>
+        <v>1.79742E7</v>
       </c>
     </row>
     <row r="3">
@@ -116,13 +116,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C3" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>4.07036E7</v>
+        <v>2478200.0</v>
       </c>
     </row>
     <row r="4">
@@ -130,13 +130,13 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C4" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>4.638378E7</v>
+        <v>5491200.0</v>
       </c>
     </row>
     <row r="5">
@@ -144,13 +144,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C5" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>3.437449E8</v>
+        <v>7978300.0</v>
       </c>
     </row>
     <row r="6">
@@ -158,13 +158,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C6" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>3.4291622E8</v>
+        <v>6108500.0</v>
       </c>
     </row>
     <row r="7">
@@ -172,13 +172,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C7" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>3.5122836E8</v>
+        <v>8409600.0</v>
       </c>
     </row>
     <row r="8">
@@ -186,13 +186,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C8" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>1.285362E7</v>
+        <v>5.776E7</v>
       </c>
     </row>
     <row r="9">
@@ -200,13 +200,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C9" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>7041560.0</v>
+        <v>4.04369E7</v>
       </c>
     </row>
     <row r="10">
@@ -214,13 +214,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C10" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>2.157416E7</v>
+        <v>4.12409E7</v>
       </c>
     </row>
     <row r="11">
@@ -228,13 +228,13 @@
         <v>5</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C11" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>3229440.0</v>
+        <v>4.5423E7</v>
       </c>
     </row>
     <row r="12">
@@ -242,13 +242,13 @@
         <v>5</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C12" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>6560880.0</v>
+        <v>1249000.0</v>
       </c>
     </row>
     <row r="13">
@@ -256,13 +256,13 @@
         <v>5</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C13" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>3878960.0</v>
+        <v>3142000.0</v>
       </c>
     </row>
     <row r="14">
@@ -270,13 +270,13 @@
         <v>5</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C14" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>2.913706E7</v>
+        <v>2683000.0</v>
       </c>
     </row>
     <row r="15">
@@ -284,13 +284,13 @@
         <v>5</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C15" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>4.707114E7</v>
+        <v>5567600.0</v>
       </c>
     </row>
     <row r="16">
@@ -298,13 +298,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>1000.0</v>
+        <v>100.0</v>
       </c>
       <c r="C16" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>4.95406E7</v>
+        <v>1263400.0</v>
       </c>
     </row>
     <row r="17">
@@ -312,13 +312,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C17" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>1.210302E7</v>
+        <v>3899200.0</v>
       </c>
     </row>
     <row r="18">
@@ -326,13 +326,13 @@
         <v>5</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C18" t="n" s="0">
         <v>5.0</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>2001880.0</v>
+        <v>7784100.0</v>
       </c>
     </row>
     <row r="19">
@@ -340,13 +340,13 @@
         <v>5</v>
       </c>
       <c r="B19" t="n" s="0">
-        <v>10.0</v>
+        <v>1000.0</v>
       </c>
       <c r="C19" t="n" s="0">
         <v>10.0</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>3227240.0</v>
+        <v>1.23268E7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Now we store all the measured times of each run
</commit_message>
<xml_diff>
--- a/time_measurements.xlsx
+++ b/time_measurements.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="8">
   <si>
     <t>Packet Type</t>
   </si>
@@ -23,7 +23,13 @@
     <t>Nesting Level</t>
   </si>
   <si>
-    <t>Average Time (ns)</t>
+    <t>Iteration 1 Time (ns)</t>
+  </si>
+  <si>
+    <t>Iteration 2 Time (ns)</t>
+  </si>
+  <si>
+    <t>Iteration 3 Time (ns)</t>
   </si>
   <si>
     <t>json</t>
@@ -74,13 +80,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.8046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="16.48828125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="12.95703125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="17.125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="19.1875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="19.1875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="19.1875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -96,10 +104,16 @@
       <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n" s="0">
         <v>10.0</v>
@@ -108,12 +122,18 @@
         <v>1.0</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>1.79742E7</v>
+        <v>2.42128E7</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>8260900.0</v>
+      </c>
+      <c r="F2" t="n" s="0">
+        <v>7221700.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3" t="n" s="0">
         <v>10.0</v>
@@ -122,12 +142,18 @@
         <v>5.0</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>2478200.0</v>
+        <v>7629000.0</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>5708100.0</v>
+      </c>
+      <c r="F3" t="n" s="0">
+        <v>5500600.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B4" t="n" s="0">
         <v>10.0</v>
@@ -136,12 +162,18 @@
         <v>10.0</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>5491200.0</v>
+        <v>1.79629E7</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>1.63735E7</v>
+      </c>
+      <c r="F4" t="n" s="0">
+        <v>1.63022E7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n" s="0">
         <v>100.0</v>
@@ -150,12 +182,18 @@
         <v>1.0</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>7978300.0</v>
+        <v>4.44493E7</v>
+      </c>
+      <c r="E5" t="n" s="0">
+        <v>4.25293E7</v>
+      </c>
+      <c r="F5" t="n" s="0">
+        <v>4.05195E7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B6" t="n" s="0">
         <v>100.0</v>
@@ -164,12 +202,18 @@
         <v>5.0</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>6108500.0</v>
+        <v>3.88954E7</v>
+      </c>
+      <c r="E6" t="n" s="0">
+        <v>3.84408E7</v>
+      </c>
+      <c r="F6" t="n" s="0">
+        <v>3.83661E7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B7" t="n" s="0">
         <v>100.0</v>
@@ -178,12 +222,18 @@
         <v>10.0</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>8409600.0</v>
+        <v>4.31598E7</v>
+      </c>
+      <c r="E7" t="n" s="0">
+        <v>4.40892E7</v>
+      </c>
+      <c r="F7" t="n" s="0">
+        <v>4.45201E7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B8" t="n" s="0">
         <v>1000.0</v>
@@ -192,12 +242,18 @@
         <v>1.0</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>5.776E7</v>
+        <v>3.579282E8</v>
+      </c>
+      <c r="E8" t="n" s="0">
+        <v>3.900699E8</v>
+      </c>
+      <c r="F8" t="n" s="0">
+        <v>3.728683E8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B9" t="n" s="0">
         <v>1000.0</v>
@@ -206,12 +262,18 @@
         <v>5.0</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>4.04369E7</v>
+        <v>3.8657E8</v>
+      </c>
+      <c r="E9" t="n" s="0">
+        <v>3.513631E8</v>
+      </c>
+      <c r="F9" t="n" s="0">
+        <v>3.547131E8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B10" t="n" s="0">
         <v>1000.0</v>
@@ -220,12 +282,18 @@
         <v>10.0</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>4.12409E7</v>
+        <v>3.564002E8</v>
+      </c>
+      <c r="E10" t="n" s="0">
+        <v>3.643152E8</v>
+      </c>
+      <c r="F10" t="n" s="0">
+        <v>3.674636E8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B11" t="n" s="0">
         <v>10.0</v>
@@ -234,12 +302,18 @@
         <v>1.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>4.5423E7</v>
+        <v>4.21256E7</v>
+      </c>
+      <c r="E11" t="n" s="0">
+        <v>2888000.0</v>
+      </c>
+      <c r="F11" t="n" s="0">
+        <v>3262300.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B12" t="n" s="0">
         <v>10.0</v>
@@ -248,12 +322,18 @@
         <v>5.0</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>1249000.0</v>
+        <v>2909900.0</v>
+      </c>
+      <c r="E12" t="n" s="0">
+        <v>3027100.0</v>
+      </c>
+      <c r="F12" t="n" s="0">
+        <v>1572200.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B13" t="n" s="0">
         <v>10.0</v>
@@ -262,12 +342,18 @@
         <v>10.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>3142000.0</v>
+        <v>6392600.0</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>3594300.0</v>
+      </c>
+      <c r="F13" t="n" s="0">
+        <v>3933400.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B14" t="n" s="0">
         <v>100.0</v>
@@ -276,12 +362,18 @@
         <v>1.0</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>2683000.0</v>
+        <v>1.5659E7</v>
+      </c>
+      <c r="E14" t="n" s="0">
+        <v>2472400.0</v>
+      </c>
+      <c r="F14" t="n" s="0">
+        <v>2595200.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B15" t="n" s="0">
         <v>100.0</v>
@@ -290,12 +382,18 @@
         <v>5.0</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>5567600.0</v>
+        <v>6465800.0</v>
+      </c>
+      <c r="E15" t="n" s="0">
+        <v>7139600.0</v>
+      </c>
+      <c r="F15" t="n" s="0">
+        <v>5820200.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B16" t="n" s="0">
         <v>100.0</v>
@@ -304,12 +402,18 @@
         <v>10.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>1263400.0</v>
+        <v>5966300.0</v>
+      </c>
+      <c r="E16" t="n" s="0">
+        <v>3444200.0</v>
+      </c>
+      <c r="F16" t="n" s="0">
+        <v>1.36789E7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B17" t="n" s="0">
         <v>1000.0</v>
@@ -318,12 +422,18 @@
         <v>1.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>3899200.0</v>
+        <v>2.99286E7</v>
+      </c>
+      <c r="E17" t="n" s="0">
+        <v>3.09273E7</v>
+      </c>
+      <c r="F17" t="n" s="0">
+        <v>2.76777E7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B18" t="n" s="0">
         <v>1000.0</v>
@@ -332,12 +442,18 @@
         <v>5.0</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>7784100.0</v>
+        <v>4.12872E7</v>
+      </c>
+      <c r="E18" t="n" s="0">
+        <v>4.40654E7</v>
+      </c>
+      <c r="F18" t="n" s="0">
+        <v>4.54484E7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B19" t="n" s="0">
         <v>1000.0</v>
@@ -346,7 +462,13 @@
         <v>10.0</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>1.23268E7</v>
+        <v>5.61482E7</v>
+      </c>
+      <c r="E19" t="n" s="0">
+        <v>4.18286E7</v>
+      </c>
+      <c r="F19" t="n" s="0">
+        <v>5.60208E7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>